<commit_message>
Regenerated fabrication files after LED replacement.
</commit_message>
<xml_diff>
--- a/HARDWARE/KICAD/Fabrication/ColorTemp Rev.00  - PICK AND PLACE (JLCPCB).xlsx
+++ b/HARDWARE/KICAD/Fabrication/ColorTemp Rev.00  - PICK AND PLACE (JLCPCB).xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Andre\ENGINEERING\PROJECTS\MECHATRONIX LAB\ColorTemp\HARDWARE\KICAD\Fabrication\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{D15DAFCB-5351-4826-8AB8-67D49FDBDD67}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8B70D6AD-4556-4FE7-B83F-5DD8EEEE7596}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="13920" yWindow="-17505" windowWidth="21600" windowHeight="11295" xr2:uid="{11F100F3-6AEC-4872-856B-C889B232DE0C}"/>
+    <workbookView xWindow="-8295" yWindow="-16065" windowWidth="21600" windowHeight="11295" xr2:uid="{11F100F3-6AEC-4872-856B-C889B232DE0C}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -518,11 +518,11 @@
       <c r="C2">
         <v>4.5</v>
       </c>
-      <c r="D2" t="s">
-        <v>24</v>
-      </c>
-      <c r="E2">
+      <c r="D2">
         <v>180</v>
+      </c>
+      <c r="E2" t="s">
+        <v>24</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
@@ -535,11 +535,11 @@
       <c r="C3">
         <v>-5.45</v>
       </c>
-      <c r="D3" t="s">
-        <v>24</v>
-      </c>
-      <c r="E3">
-        <v>0</v>
+      <c r="D3">
+        <v>0</v>
+      </c>
+      <c r="E3" t="s">
+        <v>24</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
@@ -552,11 +552,11 @@
       <c r="C4">
         <v>-9</v>
       </c>
-      <c r="D4" t="s">
-        <v>24</v>
-      </c>
-      <c r="E4">
-        <v>0</v>
+      <c r="D4">
+        <v>0</v>
+      </c>
+      <c r="E4" t="s">
+        <v>24</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
@@ -569,11 +569,11 @@
       <c r="C5">
         <v>-10.945</v>
       </c>
-      <c r="D5" t="s">
-        <v>24</v>
-      </c>
-      <c r="E5">
+      <c r="D5">
         <v>-90</v>
+      </c>
+      <c r="E5" t="s">
+        <v>24</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
@@ -586,11 +586,11 @@
       <c r="C6">
         <v>0</v>
       </c>
-      <c r="D6" t="s">
-        <v>24</v>
-      </c>
-      <c r="E6">
-        <v>0</v>
+      <c r="D6">
+        <v>180</v>
+      </c>
+      <c r="E6" t="s">
+        <v>24</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
@@ -603,11 +603,11 @@
       <c r="C7">
         <v>10.58</v>
       </c>
-      <c r="D7" t="s">
-        <v>24</v>
-      </c>
-      <c r="E7">
+      <c r="D7">
         <v>180</v>
+      </c>
+      <c r="E7" t="s">
+        <v>24</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
@@ -620,11 +620,11 @@
       <c r="C8">
         <v>4.51</v>
       </c>
-      <c r="D8" t="s">
-        <v>24</v>
-      </c>
-      <c r="E8">
+      <c r="D8">
         <v>-90</v>
+      </c>
+      <c r="E8" t="s">
+        <v>24</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
@@ -637,11 +637,11 @@
       <c r="C9">
         <v>4.51</v>
       </c>
-      <c r="D9" t="s">
-        <v>24</v>
-      </c>
-      <c r="E9">
+      <c r="D9">
         <v>-90</v>
+      </c>
+      <c r="E9" t="s">
+        <v>24</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
@@ -654,11 +654,11 @@
       <c r="C10">
         <v>1.7</v>
       </c>
-      <c r="D10" t="s">
-        <v>24</v>
-      </c>
-      <c r="E10">
+      <c r="D10">
         <v>180</v>
+      </c>
+      <c r="E10" t="s">
+        <v>24</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
@@ -671,11 +671,11 @@
       <c r="C11">
         <v>0</v>
       </c>
-      <c r="D11" t="s">
-        <v>24</v>
-      </c>
-      <c r="E11">
+      <c r="D11">
         <v>180</v>
+      </c>
+      <c r="E11" t="s">
+        <v>24</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
@@ -688,11 +688,11 @@
       <c r="C12">
         <v>-1.7</v>
       </c>
-      <c r="D12" t="s">
-        <v>24</v>
-      </c>
-      <c r="E12">
+      <c r="D12">
         <v>180</v>
+      </c>
+      <c r="E12" t="s">
+        <v>24</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.25">
@@ -705,11 +705,11 @@
       <c r="C13">
         <v>-4.45</v>
       </c>
-      <c r="D13" t="s">
-        <v>24</v>
-      </c>
-      <c r="E13">
-        <v>0</v>
+      <c r="D13">
+        <v>0</v>
+      </c>
+      <c r="E13" t="s">
+        <v>24</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.25">
@@ -722,11 +722,11 @@
       <c r="C14">
         <v>-7.5</v>
       </c>
-      <c r="D14" t="s">
-        <v>24</v>
-      </c>
-      <c r="E14">
-        <v>0</v>
+      <c r="D14">
+        <v>0</v>
+      </c>
+      <c r="E14" t="s">
+        <v>24</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.25">
@@ -739,11 +739,11 @@
       <c r="C15">
         <v>-10</v>
       </c>
-      <c r="D15" t="s">
-        <v>24</v>
-      </c>
-      <c r="E15">
-        <v>0</v>
+      <c r="D15">
+        <v>0</v>
+      </c>
+      <c r="E15" t="s">
+        <v>24</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.25">
@@ -756,11 +756,11 @@
       <c r="C16">
         <v>-10</v>
       </c>
-      <c r="D16" t="s">
-        <v>24</v>
-      </c>
-      <c r="E16">
+      <c r="D16">
         <v>180</v>
+      </c>
+      <c r="E16" t="s">
+        <v>24</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.25">
@@ -773,11 +773,11 @@
       <c r="C17">
         <v>3.25</v>
       </c>
-      <c r="D17" t="s">
-        <v>24</v>
-      </c>
-      <c r="E17">
+      <c r="D17">
         <v>90</v>
+      </c>
+      <c r="E17" t="s">
+        <v>24</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.25">
@@ -790,11 +790,11 @@
       <c r="C18">
         <v>-3.25</v>
       </c>
-      <c r="D18" t="s">
-        <v>24</v>
-      </c>
-      <c r="E18">
+      <c r="D18">
         <v>90</v>
+      </c>
+      <c r="E18" t="s">
+        <v>24</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.25">
@@ -807,11 +807,11 @@
       <c r="C19">
         <v>-6.25</v>
       </c>
-      <c r="D19" t="s">
-        <v>24</v>
-      </c>
-      <c r="E19">
-        <v>0</v>
+      <c r="D19">
+        <v>0</v>
+      </c>
+      <c r="E19" t="s">
+        <v>24</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.25">
@@ -824,11 +824,11 @@
       <c r="C20">
         <v>-10</v>
       </c>
-      <c r="D20" t="s">
-        <v>24</v>
-      </c>
-      <c r="E20">
+      <c r="D20">
         <v>180</v>
+      </c>
+      <c r="E20" t="s">
+        <v>24</v>
       </c>
     </row>
   </sheetData>

</xml_diff>